<commit_message>
Update rollout tracker and generate data using 20260522112235 data source
</commit_message>
<xml_diff>
--- a/On Air Progress Tracker.xlsx
+++ b/On Air Progress Tracker.xlsx
@@ -7955,14 +7955,22 @@
         </is>
       </c>
       <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>On Air</t>
+        </is>
+      </c>
       <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n"/>
+      <c r="G16" s="182" t="n">
+        <v>46162</v>
+      </c>
       <c r="H16" s="17" t="n"/>
       <c r="I16" s="20" t="n">
         <v>46160</v>
       </c>
-      <c r="J16" s="17" t="n"/>
+      <c r="J16" s="182" t="n">
+        <v>46162</v>
+      </c>
       <c r="K16" s="17" t="n"/>
       <c r="L16" s="17" t="n"/>
       <c r="M16" s="17" t="n"/>
@@ -8647,7 +8655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="12.75"/>
   <cols>
     <col width="3.375" customWidth="1" style="67" min="1" max="1"/>
@@ -8826,6 +8834,11 @@
           <t>Alarm（update on May 18 15:00)</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>RFI Date</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="98" t="n">
@@ -8852,7 +8865,9 @@
         </is>
       </c>
       <c r="F3" s="13" t="n"/>
-      <c r="G3" s="13" t="n"/>
+      <c r="G3" s="13" t="n">
+        <v>46158</v>
+      </c>
       <c r="H3" s="14" t="n"/>
       <c r="I3" s="183" t="n">
         <v>46168</v>
@@ -8884,6 +8899,9 @@
           <t>HUA</t>
         </is>
       </c>
+      <c r="V3" s="177" t="n">
+        <v>46140</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="98" t="n">
@@ -8910,7 +8928,9 @@
         </is>
       </c>
       <c r="F4" s="17" t="n"/>
-      <c r="G4" s="17" t="n"/>
+      <c r="G4" s="182" t="n">
+        <v>46158</v>
+      </c>
       <c r="H4" s="17" t="n"/>
       <c r="I4" s="186" t="n">
         <v>46168</v>
@@ -8941,6 +8961,9 @@
         <is>
           <t>HUA</t>
         </is>
+      </c>
+      <c r="V4" s="177" t="n">
+        <v>46140</v>
       </c>
     </row>
     <row r="5">
@@ -9078,7 +9101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="12.75"/>
   <cols>
     <col width="3.375" customWidth="1" style="67" min="1" max="1"/>
@@ -9273,6 +9296,11 @@
           <t>Alarm</t>
         </is>
       </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>RFI Date</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="78" t="n">
@@ -10110,7 +10138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="12.75" outlineLevelRow="6"/>
   <cols>
     <col width="3.375" customWidth="1" style="67" min="1" max="1"/>
@@ -10277,6 +10305,11 @@
           <t>Alarm（update on May 18 15:00)</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>RFI Date</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="98" t="n">

</xml_diff>